<commit_message>
ADI-03: estado = dato válido (no inferido) persistido desde estado de apps; sin marca *
- base_de_datos.estado_bd completado (94) con la regla válida: BD operativa si tiene app
  operativa (también En análisis/Candidato/De baja). Ahora es dato real y aparece en el CRUD.
- Quitada la marca * del estado en ADI-03 (no es inferencia, es regla app→BD)
- Normalizado casing 'DE BAJA' -> 'De baja'

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-03.xlsx
+++ b/client/public/artefactos/ADI-03.xlsx
@@ -640,7 +640,7 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -745,7 +745,7 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -850,7 +850,7 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -955,7 +955,7 @@
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -1169,7 +1169,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1274,7 +1274,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1714,14 +1714,10 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>Producción</t>
@@ -1729,22 +1725,22 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ONPSRVPRDSQL17</t>
+          <t>ONPBDONPPR01</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>COT 4</t>
+          <t>COT 5</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Windows Server 2019 Standard</t>
+          <t>AIX 7.3</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>138644.31</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1772,17 +1768,17 @@
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Versión fuera de soporte. *</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>Fuera de alcance</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>No aplica de acuerdo al correo: "[ONP-DE_BDI] Solicitud de información pendiente - Inventarios de bases de datos / Cronograma de Reuniones para levantar información" de fecha 14-10-2026 remitido por:Jesus E. Aguirre Daza.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1807,10 +1803,14 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>Producción</t>
@@ -1818,22 +1818,22 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>ONPBDONPPR01</t>
+          <t>SRVWNPSDBPR01</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>COT 5</t>
+          <t>COT 4</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>AIX 7.3</t>
+          <t>Windows Server 2019 Standard</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>138644.31</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1867,11 +1867,7 @@
           <t>Fuera de alcance</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>No aplica de acuerdo al correo: "[ONP-DE_BDI] Solicitud de información pendiente - Inventarios de bases de datos / Cronograma de Reuniones para levantar información" de fecha 14-10-2026 remitido por:Jesus E. Aguirre Daza.</t>
-        </is>
-      </c>
+      <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1896,7 +1892,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1911,7 +1907,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SRVWNPSDBPR01</t>
+          <t>ONPSRVPRDSQL17</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1926,7 +1922,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>92</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1954,7 +1950,11 @@
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Versión fuera de soporte. *</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
           <t>Fuera de alcance</t>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -2700,7 +2700,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2914,7 +2914,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -3133,7 +3133,7 @@
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>DE BAJA</t>
+          <t>De baja</t>
         </is>
       </c>
       <c r="W37" t="inlineStr"/>
@@ -4574,7 +4574,7 @@
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
@@ -4873,7 +4873,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W43" t="inlineStr"/>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W44" t="inlineStr"/>
@@ -5467,7 +5467,7 @@
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W49" t="inlineStr"/>
@@ -5996,7 +5996,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W54" t="inlineStr"/>
@@ -6097,7 +6097,7 @@
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W55" t="inlineStr"/>
@@ -6198,7 +6198,7 @@
       <c r="U56" t="inlineStr"/>
       <c r="V56" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W56" t="inlineStr"/>
@@ -6299,7 +6299,7 @@
       <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W57" t="inlineStr"/>
@@ -6400,7 +6400,7 @@
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W58" t="inlineStr"/>
@@ -6501,7 +6501,7 @@
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W59" t="inlineStr"/>
@@ -6606,7 +6606,7 @@
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W60" t="inlineStr"/>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W61" t="inlineStr"/>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W62" t="inlineStr"/>
@@ -6937,7 +6937,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W63" t="inlineStr"/>
@@ -7050,7 +7050,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W64" t="inlineStr"/>
@@ -7256,7 +7256,7 @@
       <c r="U66" t="inlineStr"/>
       <c r="V66" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W66" t="inlineStr"/>
@@ -7434,7 +7434,7 @@
       <c r="U68" t="inlineStr"/>
       <c r="V68" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W68" t="inlineStr"/>
@@ -7535,7 +7535,7 @@
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W69" t="inlineStr"/>
@@ -7745,7 +7745,7 @@
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W71" t="inlineStr"/>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W72" t="inlineStr"/>
@@ -7956,10 +7956,14 @@
           <t>Media *</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr"/>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>En baja/candidata. *</t>
+        </is>
+      </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>Candidato / De baja *</t>
+          <t>De baja</t>
         </is>
       </c>
       <c r="W73" t="inlineStr"/>
@@ -8068,7 +8072,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W74" t="inlineStr"/>
@@ -8710,7 +8714,7 @@
       <c r="U80" t="inlineStr"/>
       <c r="V80" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W80" t="inlineStr"/>
@@ -8811,7 +8815,7 @@
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W81" t="inlineStr"/>
@@ -8981,7 +8985,7 @@
       <c r="U83" t="inlineStr"/>
       <c r="V83" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W83" t="inlineStr"/>
@@ -9421,7 +9425,7 @@
       <c r="U87" t="inlineStr"/>
       <c r="V87" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W87" t="inlineStr"/>
@@ -9736,7 +9740,7 @@
       <c r="U90" t="inlineStr"/>
       <c r="V90" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W90" t="inlineStr"/>
@@ -9833,7 +9837,7 @@
       <c r="U91" t="inlineStr"/>
       <c r="V91" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W91" t="inlineStr"/>
@@ -9934,7 +9938,7 @@
       <c r="U92" t="inlineStr"/>
       <c r="V92" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W92" t="inlineStr"/>
@@ -10031,7 +10035,7 @@
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W93" t="inlineStr"/>
@@ -10128,7 +10132,7 @@
       <c r="U94" t="inlineStr"/>
       <c r="V94" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W94" t="inlineStr"/>
@@ -10233,7 +10237,7 @@
       <c r="U95" t="inlineStr"/>
       <c r="V95" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W95" t="inlineStr"/>
@@ -10338,7 +10342,7 @@
       <c r="U96" t="inlineStr"/>
       <c r="V96" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W96" t="inlineStr"/>
@@ -10443,7 +10447,7 @@
       <c r="U97" t="inlineStr"/>
       <c r="V97" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W97" t="inlineStr">
@@ -10552,7 +10556,7 @@
       <c r="U98" t="inlineStr"/>
       <c r="V98" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W98" t="inlineStr"/>
@@ -10657,7 +10661,7 @@
       <c r="U99" t="inlineStr"/>
       <c r="V99" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W99" t="inlineStr">
@@ -10762,7 +10766,7 @@
       <c r="U100" t="inlineStr"/>
       <c r="V100" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W100" t="inlineStr"/>
@@ -11085,7 +11089,7 @@
       <c r="U103" t="inlineStr"/>
       <c r="V103" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W103" t="inlineStr"/>
@@ -11179,10 +11183,14 @@
           <t>Alta *</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr"/>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>En baja/candidata. *</t>
+        </is>
+      </c>
       <c r="V104" t="inlineStr">
         <is>
-          <t>Candidato / De baja *</t>
+          <t>Candidato a dar de baja</t>
         </is>
       </c>
       <c r="W104" t="inlineStr"/>
@@ -11279,7 +11287,7 @@
       <c r="U105" t="inlineStr"/>
       <c r="V105" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W105" t="inlineStr"/>
@@ -11380,7 +11388,7 @@
       <c r="U106" t="inlineStr"/>
       <c r="V106" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W106" t="inlineStr"/>
@@ -11477,7 +11485,7 @@
       <c r="U107" t="inlineStr"/>
       <c r="V107" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W107" t="inlineStr"/>
@@ -11683,7 +11691,7 @@
       <c r="U109" t="inlineStr"/>
       <c r="V109" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W109" t="inlineStr"/>
@@ -11857,7 +11865,7 @@
       <c r="U111" t="inlineStr"/>
       <c r="V111" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W111" t="inlineStr"/>
@@ -12387,10 +12395,14 @@
           <t>Media *</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr"/>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>En baja/candidata. *</t>
+        </is>
+      </c>
       <c r="V116" t="inlineStr">
         <is>
-          <t>Candidato / De baja *</t>
+          <t>De baja</t>
         </is>
       </c>
       <c r="W116" t="inlineStr"/>
@@ -12490,12 +12502,12 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>Versión fuera de soporte. *</t>
+          <t>Versión fuera de soporte. En baja/candidata. *</t>
         </is>
       </c>
       <c r="V117" t="inlineStr">
         <is>
-          <t>Candidato / De baja *</t>
+          <t>De baja</t>
         </is>
       </c>
       <c r="W117" t="inlineStr"/>
@@ -12705,7 +12717,7 @@
       </c>
       <c r="V119" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W119" t="inlineStr"/>
@@ -12814,7 +12826,7 @@
       </c>
       <c r="V120" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W120" t="inlineStr"/>
@@ -12923,7 +12935,7 @@
       </c>
       <c r="V121" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W121" t="inlineStr"/>
@@ -13032,7 +13044,7 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W122" t="inlineStr"/>
@@ -13141,7 +13153,7 @@
       </c>
       <c r="V123" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W123" t="inlineStr"/>
@@ -13250,7 +13262,7 @@
       </c>
       <c r="V124" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W124" t="inlineStr"/>
@@ -13359,7 +13371,7 @@
       </c>
       <c r="V125" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W125" t="inlineStr"/>
@@ -13468,7 +13480,7 @@
       </c>
       <c r="V126" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W126" t="inlineStr"/>
@@ -13577,7 +13589,7 @@
       </c>
       <c r="V127" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W127" t="inlineStr"/>
@@ -13686,7 +13698,7 @@
       </c>
       <c r="V128" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W128" t="inlineStr"/>
@@ -13795,7 +13807,7 @@
       </c>
       <c r="V129" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W129" t="inlineStr"/>
@@ -13904,7 +13916,7 @@
       </c>
       <c r="V130" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W130" t="inlineStr"/>
@@ -14013,7 +14025,7 @@
       </c>
       <c r="V131" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W131" t="inlineStr"/>
@@ -14122,7 +14134,7 @@
       </c>
       <c r="V132" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W132" t="inlineStr"/>
@@ -14231,7 +14243,7 @@
       </c>
       <c r="V133" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W133" t="inlineStr"/>
@@ -14546,7 +14558,7 @@
       </c>
       <c r="V136" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W136" t="inlineStr"/>
@@ -14655,7 +14667,7 @@
       </c>
       <c r="V137" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W137" t="inlineStr"/>
@@ -14966,7 +14978,7 @@
       <c r="U140" t="inlineStr"/>
       <c r="V140" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W140" t="inlineStr"/>
@@ -15184,7 +15196,7 @@
       </c>
       <c r="V142" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W142" t="inlineStr"/>
@@ -15293,7 +15305,7 @@
       </c>
       <c r="V143" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W143" t="inlineStr"/>
@@ -15402,7 +15414,7 @@
       </c>
       <c r="V144" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W144" t="inlineStr"/>
@@ -15511,7 +15523,7 @@
       </c>
       <c r="V145" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W145" t="inlineStr"/>
@@ -15620,7 +15632,7 @@
       </c>
       <c r="V146" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W146" t="inlineStr"/>
@@ -15729,7 +15741,7 @@
       </c>
       <c r="V147" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W147" t="inlineStr"/>
@@ -15838,7 +15850,7 @@
       </c>
       <c r="V148" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W148" t="inlineStr"/>
@@ -15947,7 +15959,7 @@
       </c>
       <c r="V149" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W149" t="inlineStr"/>
@@ -16561,7 +16573,7 @@
       </c>
       <c r="V155" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W155" t="inlineStr"/>
@@ -16779,7 +16791,7 @@
       </c>
       <c r="V157" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W157" t="inlineStr"/>
@@ -16888,7 +16900,7 @@
       </c>
       <c r="V158" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W158" t="inlineStr"/>
@@ -17106,7 +17118,7 @@
       </c>
       <c r="V160" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W160" t="inlineStr"/>
@@ -17215,7 +17227,7 @@
       </c>
       <c r="V161" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W161" t="inlineStr"/>
@@ -17542,7 +17554,7 @@
       </c>
       <c r="V164" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W164" t="inlineStr"/>
@@ -17651,7 +17663,7 @@
       </c>
       <c r="V165" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W165" t="inlineStr"/>
@@ -18196,7 +18208,7 @@
       </c>
       <c r="V170" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W170" t="inlineStr"/>
@@ -18305,7 +18317,7 @@
       </c>
       <c r="V171" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W171" t="inlineStr"/>
@@ -18406,7 +18418,7 @@
       <c r="U172" t="inlineStr"/>
       <c r="V172" t="inlineStr">
         <is>
-          <t>Operativo *</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="W172" t="inlineStr"/>

</xml_diff>

<commit_message>
ADI-03: completa Tipo de información gestionada de las 2 Oracle restantes desde el DDL
BDPRAESC (modelos/plantillas de documentos - Aescribe) y BDPRGCD (gestión de contenido
documental - FileNet GCD): su nomenclatura no matcheó el diccionario de entidades, se derivó
el tipo de info de la estructura DDL. 0 Oracle con estructura quedan sin tipo de información.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-03.xlsx
+++ b/client/public/artefactos/ADI-03.xlsx
@@ -1890,10 +1890,14 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Producción</t>
@@ -1901,33 +1905,37 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ONPBDONPPR01</t>
+          <t>SRVWNPSDBPR01</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>COT 5</t>
+          <t>COT 4</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>AIX 7.3</t>
+          <t>Windows Server 2019 Standard</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>138644.31</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>1665.67</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1961,11 +1969,7 @@
           <t>Fuera de alcance</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>No aplica de acuerdo al correo: "[ONP-DE_BDI] Solicitud de información pendiente - Inventarios de bases de datos / Cronograma de Reuniones para levantar información" de fecha 14-10-2026 remitido por:Jesus E. Aguirre Daza.</t>
-        </is>
-      </c>
+      <c r="Z14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1990,14 +1994,10 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Producción</t>
@@ -2005,37 +2005,33 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SRVWNPSDBPR01</t>
+          <t>ONPBDONPPR01</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>COT 4</t>
+          <t>COT 5</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Windows Server 2019 Standard</t>
+          <t>AIX 7.3</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.02</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>138644.31</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1665.67</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2069,7 +2065,11 @@
           <t>Fuera de alcance</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>No aplica de acuerdo al correo: "[ONP-DE_BDI] Solicitud de información pendiente - Inventarios de bases de datos / Cronograma de Reuniones para levantar información" de fecha 14-10-2026 remitido por:Jesus E. Aguirre Daza.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4600,7 +4600,11 @@
           <t>Transaccional (relacional) *</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Modelos y plantillas de documentos, marcas y productos (sistema Aescribe) *</t>
+        </is>
+      </c>
       <c r="Q36" t="inlineStr">
         <is>
           <t>Misional | Soporte</t>
@@ -5824,7 +5828,11 @@
           <t>Base de datos relacional</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Gestión de contenido documental (FileNet GCD) *</t>
+        </is>
+      </c>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr"/>
@@ -13929,7 +13937,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>BD SQL Server 2008 R2 en producción; soporta AP101; dominio Gestión Administrativa, Personal y Logística *</t>
+          <t>BD SQL Server 2022 en producción; soporta AP101; dominio Gestión Administrativa, Personal y Logística *</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13939,12 +13947,12 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2008 R2</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -13954,7 +13962,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>ONPSRVSMEF</t>
+          <t>SRVWNSMEFPR01</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -13964,12 +13972,12 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Windows server 2012 R2</t>
+          <t>Windows Server 2022 Standard</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>8.61</t>
+          <t>4.37</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -13979,7 +13987,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>938</t>
+          <t>929</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -14024,14 +14032,10 @@
           <t>Media *</t>
         </is>
       </c>
-      <c r="X117" t="inlineStr">
-        <is>
-          <t>Versión fuera de soporte. En baja/candidata. *</t>
-        </is>
-      </c>
+      <c r="X117" t="inlineStr"/>
       <c r="Y117" t="inlineStr">
         <is>
-          <t>De baja</t>
+          <t>Fuera de alcance</t>
         </is>
       </c>
       <c r="Z117" t="inlineStr"/>
@@ -14049,7 +14053,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>BD SQL Server 2022 en producción; soporta AP101; dominio Gestión Administrativa, Personal y Logística *</t>
+          <t>BD SQL Server 2008 R2 en producción; soporta AP101; dominio Gestión Administrativa, Personal y Logística *</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -14059,12 +14063,12 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2008 R2</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -14074,7 +14078,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>SRVWNSMEFPR01</t>
+          <t>ONPSRVSMEF</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -14084,12 +14088,12 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Windows Server 2022 Standard</t>
+          <t>Windows server 2012 R2</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>4.37</t>
+          <t>8.61</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -14099,7 +14103,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>929</t>
+          <t>938</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -14144,10 +14148,14 @@
           <t>Media *</t>
         </is>
       </c>
-      <c r="X118" t="inlineStr"/>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>Versión fuera de soporte. En baja/candidata. *</t>
+        </is>
+      </c>
       <c r="Y118" t="inlineStr">
         <is>
-          <t>Fuera de alcance</t>
+          <t>De baja</t>
         </is>
       </c>
       <c r="Z118" t="inlineStr"/>

</xml_diff>

<commit_message>
ADI-04: Áreas usuarias vía aplicacion_area→oficina (unificado con ADI-03)
+ F-11: 8 relaciones esquema→app y ~96 comentarios rescatados (reflejados en los artefactos
en vivo + Excel regenerado). vincula_esquemas_apps.py / rescata_todos_f11.py.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-03.xlsx
+++ b/client/public/artefactos/ADI-03.xlsx
@@ -3844,17 +3844,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Inversiones previsionales | Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales | Seguros previsionales</t>
+          <t>Acompañamiento al asegurado | Gestión Administrativa, Personal y Logística | Inversiones previsionales | Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales | Seguros previsionales</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>M1 Elección e incorporación al régimen previsional | M3 Acumulación y acreditación de aportes | M4 Reconocimiento de derechos previsionales | M5 Aseguramiento al SCTR | M9 Administración de inversiones previsionales | S1 Gestión de tecnologías de la información</t>
+          <t>M1 Elección e incorporación al régimen previsional | M11 Acompañamiento al asegurado | M3 Acumulación y acreditación de aportes | M4 Reconocimiento de derechos previsionales | M5 Aseguramiento al SCTR | M9 Administración de inversiones previsionales | S1 Gestión de tecnologías de la información | S2 Gestión de recursos humanos</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Oficina de Tecnologías de la Información · Subdirección de Afiliación y Gestión de Aportes · Subdirección de Fiscalización Previsional · Subdirección de Inversiones Inmobiliarias · Unidad de Infraestructura y Soporte Tecnológico · Unidad de Ingeniería de Software</t>
+          <t>Dirección de Gestión Previsional · Oficina de Tecnologías de la Información · Subdirección de Afiliación y Gestión de Aportes · Subdirección de Fiscalización Previsional · Subdirección de Inversiones Inmobiliarias · Unidad de Infraestructura y Soporte Tecnológico · Unidad de Ingeniería de Software</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>AP021 Módulo de Afiliación Facultativa | AP022 MAF ONLINE | AP023 Módulo de Consulta de Cuenta Individual del Asegurado al Sistema Nacional de Pensiones | AP034 Portal del SCTR | AP040 Sistema de Gestión SCTR | AP042 Sistema de Administración de Accesos | AP044 Sistema de Administración Inmobiliaria | AP062 Sistema de Parámetros y Mantenimientos Generales | AP063 SRU Registro Unificado DL 20530 | AP083 Sincroniza APP | APTEMP13 Varios</t>
+          <t>AP021 Módulo de Afiliación Facultativa | AP022 MAF ONLINE | AP023 Módulo de Consulta de Cuenta Individual del Asegurado al Sistema Nacional de Pensiones | AP034 Portal del SCTR | AP040 Sistema de Gestión SCTR | AP042 Sistema de Administración de Accesos | AP044 Sistema de Administración Inmobiliaria | AP062 Sistema de Parámetros y Mantenimientos Generales | AP063 SRU Registro Unificado DL 20530 | AP083 Sincroniza APP | APTEMP03 SHAREPOINT | APTEMP13 Varios</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
@@ -4100,17 +4100,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Gestión Administrativa, Personal y Logística | Gestión Documental y Archivo | Regímenes previsionales</t>
+          <t>Apelaciones previsionales | Gestión Administrativa, Personal y Logística | Gestión Documental y Archivo | Regímenes previsionales</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>M4 Reconocimiento de derechos previsionales | S2 Gestión de recursos humanos | S3 Gestión del abastecimiento | S4 Gestión documental | S5 Gestión financiera y contable</t>
+          <t>M3 Acumulación y acreditación de aportes | M4 Reconocimiento de derechos previsionales | M7 Gestión de apelaciones previsionales | S2 Gestión de recursos humanos | S3 Gestión del abastecimiento | S4 Gestión documental | S5 Gestión financiera y contable</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Oficina de Administración · Subdirección de Afiliación y Gestión de Aportes · Subdirección de Programación y Control Previsional</t>
+          <t>Oficina de Administración · Subdirección de Afiliación y Gestión de Aportes · Subdirección de Orientación Previsional · Subdirección de Programación y Control Previsional</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>AP043 Sistema de Archivo Central de Planillas | AP057 Sistema Integrado de Gestión Administrativa | AP060 Sistema de Consulta de Stock</t>
+          <t xml:space="preserve">AP043 Sistema de Archivo Central de Planillas | AP057 Sistema Integrado de Gestión Administrativa | AP060 Sistema de Consulta de Stock | AP069 Sistema de VIsualización Documental | AP095 </t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>AP006 Sistema de Autenticación de Usuarios | AP007 Sistema de Gestión de Claves para Instituciones | AP014 Sistema Fonahpu Power Builder | AP035 Sistema de Información ONPVIRTUAL | AP046 Sistema de Consulta de Afiliados al Sistema Privado de Pensiones | AP047 Sistema de Seguimiento de Control Interno | AP048 Sistema de Consulta de Cuenta Individual de Empleadores y Asegurados | AP049 Sistema de Consulta LIBAPO, IMT Y Resoluciones | AP051 Sistema de Seguridad de Accesos | AP052 Sistema Fonahpu Web | AP054 Sistema de Gestión de Control Plantillas | AP056 Sistema de Gestión de documentos APPENS | AP058 Sistema de Recaudación | AP071 Sistema de Servicios Zona Segura ONP | AP088 Sistema de Gestión de Claves virtuales para aportantes y pensionistas</t>
+          <t>AP006 Sistema de Autenticación de Usuarios | AP007 Sistema de Gestión de Claves para Instituciones | AP014 Sistema Fonahpu Power Builder | AP035 Sistema de Información ONPVIRTUAL | AP043 Sistema de Archivo Central de Planillas | AP046 Sistema de Consulta de Afiliados al Sistema Privado de Pensiones | AP047 Sistema de Seguimiento de Control Interno | AP048 Sistema de Consulta de Cuenta Individual de Empleadores y Asegurados | AP049 Sistema de Consulta LIBAPO, IMT Y Resoluciones | AP051 Sistema de Seguridad de Accesos | AP052 Sistema Fonahpu Web | AP054 Sistema de Gestión de Control Plantillas | AP056 Sistema de Gestión de documentos APPENS | AP058 Sistema de Recaudación | AP071 Sistema de Servicios Zona Segura ONP | AP088 Sistema de Gestión de Claves virtuales para aportantes y pensionistas</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>AP027 Nuevo Sistema de Administración de Inmuebles | AP036 PIDE | AP045 Sistema de Cálculo Actuarial | APTEMP13 Varios</t>
+          <t>AP027 Nuevo Sistema de Administración de Inmuebles | AP036 PIDE | AP045 Sistema de Cálculo Actuarial | AP097  | APTEMP13 Varios</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">

</xml_diff>

<commit_message>
SIGA: asociar SIGA_1782/SIGA_55 (x2) a AP057 operativo
Las 3 fuentes SIGA (id_bd 141/126/140, FTE-114/115/116 en ADI-03)
estaban ligadas solo a AP101 'SIGA MEF' (De Baja). Se reasignan a AP057
'Sistema Integrado de Gestión Administrativa' (Operativo, Alta, OAD, con
S5 Gestión financiera y contable + S3 Abastecimiento + S2 RR.HH.) y se
elimina la relación vieja con AP101. estado_bd -> Operativo.

Quedan con dominio 'Gestión Administrativa, Personal y Logística',
oficina 'Oficina de Administración' y criticidad Alta en ADI-03/04/07/09.
Excel descargables regenerados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-03.xlsx
+++ b/client/public/artefactos/ADI-03.xlsx
@@ -8909,7 +8909,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>ONPBMONDBP01</t>
+          <t>ONPWPSDBP01</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -8948,56 +8948,24 @@
         </is>
       </c>
       <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr">
-        <is>
-          <t>Misional | Soporte</t>
-        </is>
-      </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales</t>
-        </is>
-      </c>
-      <c r="S66" t="inlineStr">
-        <is>
-          <t>M1 Elección e incorporación al régimen previsional | S1 Gestión de tecnologías de la información</t>
-        </is>
-      </c>
-      <c r="T66" t="inlineStr">
-        <is>
-          <t>Oficina de Tecnologías de la Información · Unidad de Infraestructura y Soporte Tecnológico</t>
-        </is>
-      </c>
-      <c r="U66" t="inlineStr">
-        <is>
-          <t>CARLOS SULLON | Nelly Cardenas</t>
-        </is>
-      </c>
-      <c r="V66" t="inlineStr">
-        <is>
-          <t>NELLY CARDENAS</t>
-        </is>
-      </c>
-      <c r="W66" t="inlineStr">
-        <is>
-          <t>AP005 Sistema de Aportes y Pensionamiento | APTEMP13 Varios</t>
-        </is>
-      </c>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr"/>
+      <c r="V66" t="inlineStr"/>
+      <c r="W66" t="inlineStr"/>
       <c r="X66" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="Y66" t="inlineStr"/>
-      <c r="Z66" t="inlineStr">
-        <is>
-          <t>Alta *</t>
-        </is>
-      </c>
+      <c r="Z66" t="inlineStr"/>
       <c r="AA66" t="inlineStr"/>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>Operativo</t>
+          <t>Fuera de alcance</t>
         </is>
       </c>
       <c r="AC66" t="inlineStr"/>
@@ -9036,7 +9004,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>ONPWPSDBP01</t>
+          <t>ONPBMONDBP01</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -9075,24 +9043,56 @@
         </is>
       </c>
       <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
-      <c r="T67" t="inlineStr"/>
-      <c r="U67" t="inlineStr"/>
-      <c r="V67" t="inlineStr"/>
-      <c r="W67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Misional | Soporte</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>M1 Elección e incorporación al régimen previsional | S1 Gestión de tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Oficina de Tecnologías de la Información · Unidad de Infraestructura y Soporte Tecnológico</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>CARLOS SULLON | Nelly Cardenas</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>NELLY CARDENAS</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>AP005 Sistema de Aportes y Pensionamiento | APTEMP13 Varios</t>
+        </is>
+      </c>
       <c r="X67" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="Y67" t="inlineStr"/>
-      <c r="Z67" t="inlineStr"/>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>Alta *</t>
+        </is>
+      </c>
       <c r="AA67" t="inlineStr"/>
       <c r="AB67" t="inlineStr">
         <is>
-          <t>Fuera de alcance</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="AC67" t="inlineStr"/>
@@ -10954,7 +10954,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>v10.5.0.4</t>
+          <t>v9.5.0.9</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -10965,22 +10965,34 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>ONPBMDBP01</t>
+          <t>ONPBMONDBP01</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>COT 4</t>
+          <t>COT 5</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>AIX 7.2</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
+          <t>AIX 6.1</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>267</t>
+        </is>
+      </c>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr">
         <is>
@@ -10988,24 +11000,56 @@
         </is>
       </c>
       <c r="P82" t="inlineStr"/>
-      <c r="Q82" t="inlineStr"/>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
-      <c r="T82" t="inlineStr"/>
-      <c r="U82" t="inlineStr"/>
-      <c r="V82" t="inlineStr"/>
-      <c r="W82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Misional | Soporte</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>M1 Elección e incorporación al régimen previsional | S1 Gestión de tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Oficina de Tecnologías de la Información · Unidad de Infraestructura y Soporte Tecnológico</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>CARLOS SULLON | Nelly Cardenas</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>NELLY CARDENAS</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>AP005 Sistema de Aportes y Pensionamiento | APTEMP13 Varios</t>
+        </is>
+      </c>
       <c r="X82" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr"/>
-      <c r="Z82" t="inlineStr"/>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>Alta *</t>
+        </is>
+      </c>
       <c r="AA82" t="inlineStr"/>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>Fuera de alcance</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="AC82" t="inlineStr"/>
@@ -11033,7 +11077,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>v9.5.0.9</t>
+          <t>v10.5.0.4</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -11044,34 +11088,22 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>ONPBMONDBP01</t>
+          <t>ONPBMDBP01</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>COT 5</t>
+          <t>COT 4</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>AIX 6.1</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="M83" t="inlineStr">
-        <is>
-          <t>267</t>
-        </is>
-      </c>
+          <t>AIX 7.2</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr">
         <is>
@@ -11079,56 +11111,24 @@
         </is>
       </c>
       <c r="P83" t="inlineStr"/>
-      <c r="Q83" t="inlineStr">
-        <is>
-          <t>Misional | Soporte</t>
-        </is>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales</t>
-        </is>
-      </c>
-      <c r="S83" t="inlineStr">
-        <is>
-          <t>M1 Elección e incorporación al régimen previsional | S1 Gestión de tecnologías de la información</t>
-        </is>
-      </c>
-      <c r="T83" t="inlineStr">
-        <is>
-          <t>Oficina de Tecnologías de la Información · Unidad de Infraestructura y Soporte Tecnológico</t>
-        </is>
-      </c>
-      <c r="U83" t="inlineStr">
-        <is>
-          <t>CARLOS SULLON | Nelly Cardenas</t>
-        </is>
-      </c>
-      <c r="V83" t="inlineStr">
-        <is>
-          <t>NELLY CARDENAS</t>
-        </is>
-      </c>
-      <c r="W83" t="inlineStr">
-        <is>
-          <t>AP005 Sistema de Aportes y Pensionamiento | APTEMP13 Varios</t>
-        </is>
-      </c>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr"/>
+      <c r="U83" t="inlineStr"/>
+      <c r="V83" t="inlineStr"/>
+      <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr"/>
-      <c r="Z83" t="inlineStr">
-        <is>
-          <t>Alta *</t>
-        </is>
-      </c>
+      <c r="Z83" t="inlineStr"/>
       <c r="AA83" t="inlineStr"/>
       <c r="AB83" t="inlineStr">
         <is>
-          <t>Operativo</t>
+          <t>Fuera de alcance</t>
         </is>
       </c>
       <c r="AC83" t="inlineStr"/>
@@ -14495,7 +14495,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>v10.1.0.5</t>
+          <t>v10.5.0.8</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -14506,7 +14506,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>ONPODMCBDP01</t>
+          <t>ONPODMSBDP01</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -14521,7 +14521,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>453.46</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -14531,38 +14531,70 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>156</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
         <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Transaccional (relacional) *</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr"/>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Misional | Soporte</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>M1 Elección e incorporación al régimen previsional | S1 Gestión de tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>Oficina de Tecnologías de la Información · Unidad de Infraestructura y Soporte Tecnológico</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>CARLOS SULLON | Nelly Cardenas</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>NELLY CARDENAS</t>
+        </is>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>AP005 Sistema de Aportes y Pensionamiento | APTEMP13 Varios</t>
+        </is>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O110" t="inlineStr">
-        <is>
-          <t>Transaccional (relacional) *</t>
-        </is>
-      </c>
-      <c r="P110" t="inlineStr"/>
-      <c r="Q110" t="inlineStr"/>
-      <c r="R110" t="inlineStr"/>
-      <c r="S110" t="inlineStr"/>
-      <c r="T110" t="inlineStr"/>
-      <c r="U110" t="inlineStr"/>
-      <c r="V110" t="inlineStr"/>
-      <c r="W110" t="inlineStr"/>
-      <c r="X110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Y110" t="inlineStr"/>
-      <c r="Z110" t="inlineStr"/>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>Alta *</t>
+        </is>
+      </c>
       <c r="AA110" t="inlineStr"/>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>Fuera de alcance</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="AC110" t="inlineStr"/>
@@ -14590,7 +14622,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>v10.5.0.8</t>
+          <t>v10.1.0.5</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -14601,7 +14633,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>ONPODMSBDP01</t>
+          <t>ONPODMCBDP01</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -14616,7 +14648,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>453.46</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -14626,12 +14658,12 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>235</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -14640,56 +14672,24 @@
         </is>
       </c>
       <c r="P111" t="inlineStr"/>
-      <c r="Q111" t="inlineStr">
-        <is>
-          <t>Misional | Soporte</t>
-        </is>
-      </c>
-      <c r="R111" t="inlineStr">
-        <is>
-          <t>Plataforma, Seguridad e Interoperabilidad | Regímenes previsionales</t>
-        </is>
-      </c>
-      <c r="S111" t="inlineStr">
-        <is>
-          <t>M1 Elección e incorporación al régimen previsional | S1 Gestión de tecnologías de la información</t>
-        </is>
-      </c>
-      <c r="T111" t="inlineStr">
-        <is>
-          <t>Oficina de Tecnologías de la Información · Unidad de Infraestructura y Soporte Tecnológico</t>
-        </is>
-      </c>
-      <c r="U111" t="inlineStr">
-        <is>
-          <t>CARLOS SULLON | Nelly Cardenas</t>
-        </is>
-      </c>
-      <c r="V111" t="inlineStr">
-        <is>
-          <t>NELLY CARDENAS</t>
-        </is>
-      </c>
-      <c r="W111" t="inlineStr">
-        <is>
-          <t>AP005 Sistema de Aportes y Pensionamiento | APTEMP13 Varios</t>
-        </is>
-      </c>
+      <c r="Q111" t="inlineStr"/>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr"/>
+      <c r="T111" t="inlineStr"/>
+      <c r="U111" t="inlineStr"/>
+      <c r="V111" t="inlineStr"/>
+      <c r="W111" t="inlineStr"/>
       <c r="X111" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="Y111" t="inlineStr"/>
-      <c r="Z111" t="inlineStr">
-        <is>
-          <t>Alta *</t>
-        </is>
-      </c>
+      <c r="Z111" t="inlineStr"/>
       <c r="AA111" t="inlineStr"/>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>Operativo</t>
+          <t>Fuera de alcance</t>
         </is>
       </c>
       <c r="AC111" t="inlineStr"/>
@@ -15262,7 +15262,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>BD SQL Server 2022 en producción; soporta AP101; dominio Gestión Administrativa, Personal y Logística *</t>
+          <t>BD SQL Server 2022 en producción; soporta AP057; dominio Gestión Administrativa, Personal y Logística *</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -15326,7 +15326,7 @@
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>S5 Gestión financiera y contable</t>
+          <t>S2 Gestión de recursos humanos | S3 Gestión del abastecimiento | S5 Gestión financiera y contable</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -15334,11 +15334,19 @@
           <t>Oficina de Administración</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr"/>
-      <c r="V116" t="inlineStr"/>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>Patricia Vivas</t>
+        </is>
+      </c>
+      <c r="V116" t="inlineStr">
+        <is>
+          <t>Rosario Sonco / Marco Puente Arnao / Jose Silva / Brandy Zavala / Jenifer Cipra / Liseth Gomez / Mario Ganoza</t>
+        </is>
+      </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>AP101 SIGA MEF</t>
+          <t>AP057 Sistema Integrado de Gestión Administrativa</t>
         </is>
       </c>
       <c r="X116" t="inlineStr">
@@ -15352,14 +15360,10 @@
           <t>Media *</t>
         </is>
       </c>
-      <c r="AA116" t="inlineStr">
-        <is>
-          <t>En baja/candidata. *</t>
-        </is>
-      </c>
+      <c r="AA116" t="inlineStr"/>
       <c r="AB116" t="inlineStr">
         <is>
-          <t>De baja</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="AC116" t="inlineStr"/>
@@ -15377,7 +15381,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>BD SQL Server 2022 en producción; soporta AP101; dominio Gestión Administrativa, Personal y Logística *</t>
+          <t>BD SQL Server 2022 en producción; soporta AP057; dominio Gestión Administrativa, Personal y Logística *</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -15453,7 +15457,7 @@
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>S5 Gestión financiera y contable</t>
+          <t>S2 Gestión de recursos humanos | S3 Gestión del abastecimiento | S5 Gestión financiera y contable</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -15461,11 +15465,19 @@
           <t>Oficina de Administración</t>
         </is>
       </c>
-      <c r="U117" t="inlineStr"/>
-      <c r="V117" t="inlineStr"/>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>Patricia Vivas</t>
+        </is>
+      </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>Rosario Sonco / Marco Puente Arnao / Jose Silva / Brandy Zavala / Jenifer Cipra / Liseth Gomez / Mario Ganoza</t>
+        </is>
+      </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>AP101 SIGA MEF</t>
+          <t>AP057 Sistema Integrado de Gestión Administrativa</t>
         </is>
       </c>
       <c r="X117" t="inlineStr">
@@ -15482,7 +15494,7 @@
       <c r="AA117" t="inlineStr"/>
       <c r="AB117" t="inlineStr">
         <is>
-          <t>Fuera de alcance</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="AC117" t="inlineStr"/>
@@ -15500,7 +15512,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>BD SQL Server 2008 R2 en producción; soporta AP101; dominio Gestión Administrativa, Personal y Logística *</t>
+          <t>BD SQL Server 2008 R2 en producción; soporta AP057; dominio Gestión Administrativa, Personal y Logística *</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -15576,7 +15588,7 @@
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>S5 Gestión financiera y contable</t>
+          <t>S2 Gestión de recursos humanos | S3 Gestión del abastecimiento | S5 Gestión financiera y contable</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -15584,11 +15596,19 @@
           <t>Oficina de Administración</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr"/>
-      <c r="V118" t="inlineStr"/>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>Patricia Vivas</t>
+        </is>
+      </c>
+      <c r="V118" t="inlineStr">
+        <is>
+          <t>Rosario Sonco / Marco Puente Arnao / Jose Silva / Brandy Zavala / Jenifer Cipra / Liseth Gomez / Mario Ganoza</t>
+        </is>
+      </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>AP101 SIGA MEF</t>
+          <t>AP057 Sistema Integrado de Gestión Administrativa</t>
         </is>
       </c>
       <c r="X118" t="inlineStr">
@@ -15604,12 +15624,12 @@
       </c>
       <c r="AA118" t="inlineStr">
         <is>
-          <t>Versión fuera de soporte. En baja/candidata. *</t>
+          <t>Versión fuera de soporte. *</t>
         </is>
       </c>
       <c r="AB118" t="inlineStr">
         <is>
-          <t>De baja</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="AC118" t="inlineStr"/>

</xml_diff>